<commit_message>
Update all docs: e平屋net (Lib Work) closed on 2026/1/31
Critical market change: The only competing hiraya-specialized portal
in Japan (e平屋net by Lib Work) was shut down on January 31, 2026.
Payhome is now Japan's ONLY hiraya-specialized platform with ZERO
competitors in this niche.

Strategic implications updated across all docs:
- No geographic restrictions in Kyushu (Fukuoka/Kumamoto/Saga/Oita now open)
- e平屋net's closure validates that simple listing approach doesn't work
- Payhome's YouTube + AI + data approach is the correct differentiation
- "Japan's first AND only" positioning strengthened

Files updated:
- BUSINESS_STRATEGY.md/EN: Competitive analysis, risk section, expansion strategy
- 00_CURRENT_ISSUES.md/EN: Market positioning context
- youtube_research.md: Lib Work competitor analysis + lessons learned
- HANDOVER.md: Market context for engineers
- YouTube・SNS戦略管理.xlsx: Competitor analysis sheet

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/06_YouTube・SNS戦略/YouTube・SNS戦略管理.xlsx
+++ b/docs/06_YouTube・SNS戦略/YouTube・SNS戦略管理.xlsx
@@ -120,7 +120,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -142,11 +142,55 @@
         <color rgb="00D5D8DC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D5D8DC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D5D8DC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D5D8DC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D5D8DC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D5D8DC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D5D8DC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D5D8DC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D5D8DC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -240,6 +284,8 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -628,6 +674,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -689,6 +736,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
@@ -1000,6 +1048,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
@@ -1153,6 +1202,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -1592,6 +1642,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -1810,6 +1861,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -2015,6 +2067,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
@@ -2047,6 +2100,8 @@
           <t>最大10文字。短いほど良い</t>
         </is>
       </c>
+      <c r="C16" s="39" t="n"/>
+      <c r="D16" s="40" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="26" t="inlineStr">
@@ -2059,6 +2114,8 @@
           <t>2色以内。白＋オレンジ or 白＋黒</t>
         </is>
       </c>
+      <c r="C17" s="39" t="n"/>
+      <c r="D17" s="40" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="24" t="inlineStr">
@@ -2071,6 +2128,8 @@
           <t>太いゴシック体。角ゴシック推奨</t>
         </is>
       </c>
+      <c r="C18" s="39" t="n"/>
+      <c r="D18" s="40" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="26" t="inlineStr">
@@ -2083,6 +2142,8 @@
           <t>物件の最も映えるアングル1枚。広角</t>
         </is>
       </c>
+      <c r="C19" s="39" t="n"/>
+      <c r="D19" s="40" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="24" t="inlineStr">
@@ -2095,6 +2156,8 @@
           <t>驚き顔or指差し。表情は大げさに</t>
         </is>
       </c>
+      <c r="C20" s="39" t="n"/>
+      <c r="D20" s="40" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="26" t="inlineStr">
@@ -2107,6 +2170,8 @@
           <t>金額・坪数を大きく表示</t>
         </is>
       </c>
+      <c r="C21" s="39" t="n"/>
+      <c r="D21" s="40" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="24" t="inlineStr">
@@ -2119,7 +2184,10 @@
           <t>文字詰め込みすぎ×、背景ごちゃごちゃ×</t>
         </is>
       </c>
-    </row>
+      <c r="C22" s="39" t="n"/>
+      <c r="D22" s="40" t="n"/>
+    </row>
+    <row r="23"/>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
@@ -2284,7 +2352,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R100"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2314,6 +2382,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -3126,93 +3195,6 @@
       <c r="Q13" s="20" t="inlineStr"/>
       <c r="R13" s="20" t="inlineStr"/>
     </row>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
   </sheetData>
   <autoFilter ref="A3:R100"/>
   <mergeCells count="1">
@@ -3237,7 +3219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3261,6 +3243,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -4243,83 +4226,6 @@
       <c r="K23" s="20" t="inlineStr"/>
       <c r="L23" s="20" t="inlineStr"/>
     </row>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
   </sheetData>
   <autoFilter ref="A3:L100"/>
   <mergeCells count="1">
@@ -4341,7 +4247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J200"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -4363,6 +4269,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -4546,6 +4453,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
@@ -5051,6 +4959,8 @@
           <t>#平屋 #平屋暮らし #平屋の家 #ルームツアー #注文住宅 #マイホーム</t>
         </is>
       </c>
+      <c r="C32" s="39" t="n"/>
+      <c r="D32" s="40" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="24" t="inlineStr">
@@ -5063,6 +4973,8 @@
           <t>#鹿児島 #鹿児島住宅 #九州住宅 #鹿児島工務店 #鹿児島注文住宅</t>
         </is>
       </c>
+      <c r="C33" s="39" t="n"/>
+      <c r="D33" s="40" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="24" t="inlineStr">
@@ -5075,6 +4987,8 @@
           <t>#平屋間取り #家事動線 #中庭のある家 #回遊動線 #ランドリールーム</t>
         </is>
       </c>
+      <c r="C34" s="39" t="n"/>
+      <c r="D34" s="40" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
@@ -5087,172 +5001,9 @@
           <t>#家づくり #新築 #間取り #住宅ローン #住まい #おうち時間</t>
         </is>
       </c>
-    </row>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
+      <c r="C35" s="39" t="n"/>
+      <c r="D35" s="40" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="B33:D33"/>
@@ -5307,6 +5058,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -6312,6 +6064,7 @@
       <c r="K56" s="21" t="n"/>
       <c r="L56" s="21" t="n"/>
     </row>
+    <row r="57"/>
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="14" t="inlineStr">
         <is>
@@ -6657,6 +6410,7 @@
       </c>
       <c r="L71" s="31" t="n"/>
     </row>
+    <row r="72"/>
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="14" t="inlineStr">
         <is>
@@ -6802,6 +6556,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -6987,6 +6742,7 @@
       </c>
       <c r="F9" s="34" t="inlineStr"/>
     </row>
+    <row r="10"/>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
@@ -7926,6 +7682,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="14" t="inlineStr">
         <is>
@@ -7957,6 +7714,7 @@
           <t>ルームツアー12〜18分、後悔系8〜12分、比較系10〜15分</t>
         </is>
       </c>
+      <c r="C46" s="40" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="24" t="inlineStr">
@@ -7969,6 +7727,7 @@
           <t>金曜18:00 or 土曜10:00（視聴者のアクティブ時間）</t>
         </is>
       </c>
+      <c r="C47" s="40" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="24" t="inlineStr">
@@ -7981,6 +7740,7 @@
           <t>最初3行に要約＋CTA。チャプター付き。関連動画リンク</t>
         </is>
       </c>
+      <c r="C48" s="40" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="24" t="inlineStr">
@@ -7993,6 +7753,7 @@
           <t>次の動画への誘導＋チャンネル登録ボタン</t>
         </is>
       </c>
+      <c r="C49" s="40" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="24" t="inlineStr">
@@ -8005,6 +7766,7 @@
           <t>質問を促す。「あなたの平屋の不安は？コメントで教えて」</t>
         </is>
       </c>
+      <c r="C50" s="40" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="24" t="inlineStr">
@@ -8017,6 +7779,7 @@
           <t>動画中盤に関連動画カードを挿入（離脱防止）</t>
         </is>
       </c>
+      <c r="C51" s="40" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -8058,6 +7821,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -8099,6 +7863,7 @@
           <t>「えっ...」「やばい...」「これ見て」</t>
         </is>
       </c>
+      <c r="D5" s="40" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
@@ -8116,7 +7881,7 @@
           <t>テキストで「25坪の平屋」と表示</t>
         </is>
       </c>
-      <c r="D6" s="28" t="n"/>
+      <c r="D6" s="40" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="24" t="inlineStr">
@@ -8134,6 +7899,7 @@
           <t>飽きさせない。動きを止めない</t>
         </is>
       </c>
+      <c r="D7" s="40" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="26" t="inlineStr">
@@ -8151,7 +7917,7 @@
           <t>完視聴率が再生数に直結</t>
         </is>
       </c>
-      <c r="D8" s="28" t="n"/>
+      <c r="D8" s="40" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="24" t="inlineStr">
@@ -8169,6 +7935,7 @@
           <t>音なしでも伝わるように</t>
         </is>
       </c>
+      <c r="D9" s="40" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="26" t="inlineStr">
@@ -8186,7 +7953,7 @@
           <t>「フォローで平屋情報GET」</t>
         </is>
       </c>
-      <c r="D10" s="28" t="n"/>
+      <c r="D10" s="40" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="24" t="inlineStr">
@@ -8204,7 +7971,9 @@
           <t>量が質を生む。テストの母数を増やす</t>
         </is>
       </c>
-    </row>
+      <c r="D11" s="40" t="n"/>
+    </row>
+    <row r="12"/>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
@@ -8388,6 +8157,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
@@ -8429,6 +8199,7 @@
           <t>10物件×2本</t>
         </is>
       </c>
+      <c r="D25" s="40" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="24" t="inlineStr">
@@ -8446,6 +8217,7 @@
           <t>20本×5万=100万</t>
         </is>
       </c>
+      <c r="D26" s="40" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="24" t="inlineStr">
@@ -8463,6 +8235,7 @@
           <t>20%がバズる想定</t>
         </is>
       </c>
+      <c r="D27" s="40" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="24" t="inlineStr">
@@ -8480,6 +8253,7 @@
           <t>20本×3万=60万（ロングと合わせて100万）</t>
         </is>
       </c>
+      <c r="D28" s="40" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -8493,8 +8267,8 @@
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
     <mergeCell ref="A13:D13"/>
-    <mergeCell ref="C28:D28"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C26:D26"/>
     <mergeCell ref="C8:D8"/>
@@ -8530,6 +8304,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>

</xml_diff>